<commit_message>
corrected logic for multiple logo placement
</commit_message>
<xml_diff>
--- a/testing/test.xlsx
+++ b/testing/test.xlsx
@@ -424,9 +424,6 @@
       <c r="H1" t="str">
         <v>Supplier Name</v>
       </c>
-      <c r="I1" t="str">
-        <v>Custom Logo Size_x000d_</v>
-      </c>
       <c r="J1" t="str">
         <v/>
       </c>
@@ -478,32 +475,29 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>41432A5282</v>
+        <v>41432A5279</v>
       </c>
       <c r="B2" t="str">
-        <v>CT89240105</v>
+        <v>96000</v>
       </c>
       <c r="C2" t="str">
-        <v>Carhartt Brown</v>
+        <v>Blacktop</v>
       </c>
       <c r="D2" t="str">
-        <v>9953285_11845694</v>
+        <v>9953285_11845693</v>
       </c>
       <c r="E2" t="str">
-        <v>White</v>
+        <v xml:space="preserve">Black </v>
       </c>
       <c r="F2" t="str">
-        <v>BAG-FRONT</v>
+        <v>BAG-ON-POCKET</v>
       </c>
       <c r="G2" t="str">
-        <v>L152FNavy-10036294_11952739-72-8-9jpg</v>
+        <v>EB510FCobaltBlue-10036294_11952739-57-8-9.jpg</v>
       </c>
       <c r="H2" t="str">
         <v>SanMar</v>
       </c>
-      <c r="I2" t="str">
-        <v>100x80_x000d_</v>
-      </c>
       <c r="J2" t="str">
         <v/>
       </c>
@@ -551,6 +545,9 @@
       </c>
       <c r="Y2" t="str">
         <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v>_x000d_</v>
       </c>
     </row>
     <row r="3">
@@ -561,7 +558,7 @@
         <v>96000</v>
       </c>
       <c r="C3" t="str">
-        <v>SignalRed</v>
+        <v>Tarmac Grey Heather</v>
       </c>
       <c r="D3" t="str">
         <v>9953285_11845694</v>
@@ -570,17 +567,14 @@
         <v>White</v>
       </c>
       <c r="F3" t="str">
-        <v>BAG-FRONT</v>
+        <v>ON BAG POCKET</v>
       </c>
       <c r="G3" t="str">
-        <v>CSV40FNavy-10036294_11952742-16-8-9.jpg</v>
+        <v>EB510FDeepBlack-10036294_11952739-57-8-9.jpg</v>
       </c>
       <c r="H3" t="str">
         <v>SanMar</v>
       </c>
-      <c r="I3" t="str">
-        <v>100x80_x000d_</v>
-      </c>
       <c r="J3" t="str">
         <v/>
       </c>
@@ -634,7 +628,52 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
         <v/>
       </c>
     </row>

</xml_diff>